<commit_message>
harden credit report templates and audits
</commit_message>
<xml_diff>
--- a/skill/corporate-credit-investigation-cn/assets/流动资金类贷款授信额度测算表.xlsx
+++ b/skill/corporate-credit-investigation-cn/assets/流动资金类贷款授信额度测算表.xlsx
@@ -1565,7 +1565,7 @@
         <f>IF(C9=0,"",(D9-C9)/C9)</f>
         <v/>
       </c>
-      <c r="E12" s="16" t="n"/>
+      <c r="E12" s="58" t="n"/>
       <c r="F12" s="44" t="inlineStr">
         <is>
           <t>最近一期增长率计算=(当期累计的销售收入*12/已有期数-上年销售额)/上年销售额，或=(当期累计销售-去年同期销售)/去年同期销售，供参考</t>
@@ -1864,7 +1864,7 @@
       <c r="H23" s="45" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="18">
     <mergeCell ref="F20:H20"/>
     <mergeCell ref="F16:H16"/>

</xml_diff>